<commit_message>
terminé los cambios en reporte venta joyería, nuevo modelo
</commit_message>
<xml_diff>
--- a/Proveedores/Proveedores_joyeria_Carlos.xlsx
+++ b/Proveedores/Proveedores_joyeria_Carlos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Proveedores\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Proveedores\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -86,10 +86,10 @@
     <t>NOMBRE_NUEVO</t>
   </si>
   <si>
-    <t>CHINA</t>
-  </si>
-  <si>
     <t>PROVEEDOR</t>
+  </si>
+  <si>
+    <t>YIWU YUHANG (CHINA)</t>
   </si>
 </sst>
 </file>
@@ -110,7 +110,7 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -120,12 +120,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB1A0C7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -200,7 +194,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,7 +484,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
         <v>19</v>
@@ -549,7 +543,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:2">

</xml_diff>

<commit_message>
nuevo reporte de joyería acumulada en proceso
</commit_message>
<xml_diff>
--- a/Proveedores/Proveedores_joyeria_Carlos.xlsx
+++ b/Proveedores/Proveedores_joyeria_Carlos.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6310"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6315"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>SUCCESSFUL BOXES S.R.L.</t>
   </si>
   <si>
-    <t>SB (FABRICA)</t>
-  </si>
-  <si>
     <t>NOMBRE_NUEVO</t>
   </si>
   <si>
@@ -90,6 +87,9 @@
   </si>
   <si>
     <t>YIWU YUHANG (CHINA)</t>
+  </si>
+  <si>
+    <t>CHINA</t>
   </si>
 </sst>
 </file>
@@ -476,18 +476,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="53.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -543,7 +543,7 @@
         <v>12</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -567,7 +567,7 @@
         <v>17</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
arreglos en reporte de ventas joyería histórico
</commit_message>
<xml_diff>
--- a/Proveedores/Proveedores_joyeria_Carlos.xlsx
+++ b/Proveedores/Proveedores_joyeria_Carlos.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Proveedores\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Proveedores\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6315"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6320"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>DE CUSATIS FLAVIO A Y DE CUSATIS VALERIOL C SOC DE HECHO</t>
   </si>
@@ -475,11 +475,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="53.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -570,6 +570,14 @@
         <v>21</v>
       </c>
     </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
reporte histórico joyería de quincena. Comencé a cambiar scripts para tener dataframe de base para el resto
</commit_message>
<xml_diff>
--- a/Proveedores/Proveedores_joyeria_Carlos.xlsx
+++ b/Proveedores/Proveedores_joyeria_Carlos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>DE CUSATIS FLAVIO A Y DE CUSATIS VALERIOL C SOC DE HECHO</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>CHINA</t>
+  </si>
+  <si>
+    <t>PASSA DISEGNI S.R.L.</t>
   </si>
 </sst>
 </file>
@@ -475,7 +478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="53.453125" bestFit="1" customWidth="1"/>
@@ -508,73 +511,81 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B12" s="4" t="s">
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
inicios nueva tablero Carlos. Modificación para horas no trabajdas en gris en Tickets por hora
</commit_message>
<xml_diff>
--- a/Proveedores/Proveedores_joyeria_Carlos.xlsx
+++ b/Proveedores/Proveedores_joyeria_Carlos.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\Valeria\Reportes\Proveedores\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maval\Documents\Vale laburo\Castelli\Reportes\Proveedores\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6320"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6324"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="24">
   <si>
     <t>DE CUSATIS FLAVIO A Y DE CUSATIS VALERIOL C SOC DE HECHO</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>PASSA DISEGNI S.R.L.</t>
+  </si>
+  <si>
+    <t>PASSA DISEGNI S.R.L</t>
   </si>
 </sst>
 </file>
@@ -478,11 +481,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="53.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="53.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -519,73 +522,81 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="4" t="s">
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>